<commit_message>
Replace only matched substrings during redaction
The executor previously overwrote the entire cell or paragraph,
discarding text outside the matched alias. Use the matched
original_value substring (via replace_in_cell / replace_text) so
surrounding content is preserved, and skip sites whose original
text no longer exists in the document.
</commit_message>
<xml_diff>
--- a/examples/天齐锂业2026年半年度利润表_脱敏.xlsx
+++ b/examples/天齐锂业2026年半年度利润表_脱敏.xlsx
@@ -572,9 +572,8 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
-        <v>[公司A]</v>
-        <is>
-          <t>天齐锂业股份有限公司</t>
+        <is>
+          <t>[公司A]​‌‌​​​‌‌​‌‌​‌​​​​‌‌​​‌​‌​‌‌​‌‌‌​​‌‌‌‌​​​​‌‌​‌​​‌​‌‌​‌‌‌​​​‌​‌‌‌​​‌‌​‌‌​‌​‌‌​​​​‌​‌‌‌‌‌​​​​‌‌​​‌​​​‌‌​​​​​​‌‌​​‌​​​‌‌​‌‌​​​‌​‌‌​‌​​‌‌​​​​​​‌‌‌​​‌​​‌​‌‌​‌​​‌‌​​​‌​​‌‌​​​​​‌​‌​‌​​​​‌‌​​​‌​​‌‌​‌‌​​​‌‌‌​‌​​​‌‌​​‌‌​​‌‌​​‌‌​​‌‌‌​‌​​​‌‌​​​​​​‌‌​‌‌​​‌‌‌‌‌​​​​‌‌​​​‌​‌‌​​‌​​​‌‌​​​​‌​​‌‌‌​​‌​‌‌​​​​‌​​‌‌​‌‌‌​‌‌​​​‌‌​​‌‌​‌​‌​​‌‌​‌‌‌​​‌‌​​​​​‌‌​​​‌​​‌‌​​‌​‌​‌‌​​​‌‌​​‌‌​‌‌​​​‌‌​‌‌‌​​‌‌​​‌​</t>
         </is>
       </c>
     </row>
@@ -1147,9 +1146,8 @@
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="20" t="inlineStr">
-        <v>[公司B]</v>
-        <is>
-          <t>数据来源：天齐锂业2026年半年度报告（披露日期：2026年8月27日）。</t>
+        <is>
+          <t>数据来源：[公司B]2026年半年度报告（披露日期：2026年8月27日）。</t>
         </is>
       </c>
     </row>

</xml_diff>